<commit_message>
WNBA combo props: team/opp display, hit rate, modal chart, API slim keys
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-28.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-28.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="E3" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="F3" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G3" t="n">
-        <v>51.6</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="4">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E5" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F5" t="n">
         <v>38</v>
       </c>
       <c r="G5" t="n">
-        <v>62</v>
+        <v>61.6</v>
       </c>
     </row>
     <row r="6">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>498</v>
+        <v>517</v>
       </c>
       <c r="E8" t="n">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="F8" t="n">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="G8" t="n">
-        <v>35.5</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="9">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E10" t="n">
         <v>147</v>
       </c>
       <c r="F10" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G10" t="n">
-        <v>72.09999999999999</v>
+        <v>71.7</v>
       </c>
     </row>
     <row r="11">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E12" t="n">
         <v>108</v>
       </c>
       <c r="F12" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G12" t="n">
-        <v>66.3</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="13">
@@ -1215,16 +1215,16 @@
         <v>74</v>
       </c>
       <c r="F3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G3" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H3" t="n">
-        <v>40.7</v>
+        <v>40.2</v>
       </c>
       <c r="I3" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J3" t="n">
         <v>23.5</v>
@@ -1394,10 +1394,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>83.3</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
         <v>78.59999999999999</v>
@@ -1412,10 +1412,10 @@
         <v>9</v>
       </c>
       <c r="H5" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -1454,22 +1454,22 @@
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>75</v>
+        <v>56.5</v>
       </c>
       <c r="Y5" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="Z5" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="AA5" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="AB5" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="AC5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1540,10 +1540,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>72.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="C7" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D7" t="n">
         <v>57.7</v>
@@ -1552,10 +1552,10 @@
         <v>537</v>
       </c>
       <c r="F7" t="n">
-        <v>66.3</v>
+        <v>66.7</v>
       </c>
       <c r="G7" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H7" t="n">
         <v>47.5</v>
@@ -1606,22 +1606,22 @@
         <v>41</v>
       </c>
       <c r="X7" t="n">
-        <v>35.5</v>
+        <v>36.2</v>
       </c>
       <c r="Y7" t="n">
-        <v>498</v>
+        <v>517</v>
       </c>
       <c r="Z7" t="n">
-        <v>51.6</v>
+        <v>52.4</v>
       </c>
       <c r="AA7" t="n">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="AB7" t="n">
-        <v>62</v>
+        <v>61.6</v>
       </c>
       <c r="AC7" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AD7" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Daily slate 2026-05-30 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-28.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-28.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F2" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="G2" t="n">
-        <v>24.6</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>168</v>
+        <v>199</v>
       </c>
       <c r="E3" t="n">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="F3" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="G3" t="n">
-        <v>52.4</v>
+        <v>52.3</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G4" t="n">
-        <v>32.1</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E5" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F5" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G5" t="n">
-        <v>61.6</v>
+        <v>61.2</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E6" t="n">
         <v>20</v>
       </c>
       <c r="F6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G6" t="n">
-        <v>48.8</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="7">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>517</v>
+        <v>549</v>
       </c>
       <c r="E8" t="n">
-        <v>187</v>
+        <v>220</v>
       </c>
       <c r="F8" t="n">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G8" t="n">
-        <v>36.2</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="9">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>205</v>
+        <v>248</v>
       </c>
       <c r="E10" t="n">
-        <v>147</v>
+        <v>181</v>
       </c>
       <c r="F10" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G10" t="n">
-        <v>71.7</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>537</v>
+        <v>624</v>
       </c>
       <c r="E11" t="n">
-        <v>310</v>
+        <v>355</v>
       </c>
       <c r="F11" t="n">
-        <v>227</v>
+        <v>269</v>
       </c>
       <c r="G11" t="n">
-        <v>57.7</v>
+        <v>56.9</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="E12" t="n">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="F12" t="n">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="G12" t="n">
-        <v>66.7</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="E13" t="n">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="F13" t="n">
         <v>283</v>
       </c>
       <c r="G13" t="n">
-        <v>47.5</v>
+        <v>48.1</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="E14" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="F14" t="n">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="G14" t="n">
-        <v>21.6</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>300</v>
+        <v>435</v>
       </c>
       <c r="E15" t="n">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="F15" t="n">
-        <v>243</v>
+        <v>346</v>
       </c>
       <c r="G15" t="n">
-        <v>19</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>93</v>
+        <v>162</v>
       </c>
       <c r="E16" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="F16" t="n">
-        <v>72</v>
+        <v>129</v>
       </c>
       <c r="G16" t="n">
-        <v>22.6</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2826</v>
+        <v>3031</v>
       </c>
       <c r="E17" t="n">
-        <v>547</v>
+        <v>574</v>
       </c>
       <c r="F17" t="n">
-        <v>2279</v>
+        <v>2457</v>
       </c>
       <c r="G17" t="n">
-        <v>19.4</v>
+        <v>18.9</v>
       </c>
     </row>
   </sheetData>
@@ -1154,7 +1154,7 @@
         <v>302</v>
       </c>
       <c r="R2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="S2" t="n">
         <v>50</v>
@@ -1169,7 +1169,7 @@
         <v>2</v>
       </c>
       <c r="X2" t="n">
-        <v>33.7</v>
+        <v>34.2</v>
       </c>
       <c r="Y2" t="n">
         <v>199</v>
@@ -1203,52 +1203,52 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61.3</v>
+        <v>63.3</v>
       </c>
       <c r="C3" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D3" t="n">
-        <v>56.8</v>
+        <v>55.3</v>
       </c>
       <c r="E3" t="n">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="F3" t="n">
-        <v>51</v>
+        <v>47.6</v>
       </c>
       <c r="G3" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="H3" t="n">
-        <v>40.2</v>
+        <v>43</v>
       </c>
       <c r="I3" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="J3" t="n">
-        <v>23.5</v>
+        <v>28.6</v>
       </c>
       <c r="K3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="L3" t="n">
-        <v>6.8</v>
+        <v>13.1</v>
       </c>
       <c r="M3" t="n">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="N3" t="n">
-        <v>9.4</v>
+        <v>7.5</v>
       </c>
       <c r="O3" t="n">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="P3" t="n">
-        <v>15</v>
+        <v>14.6</v>
       </c>
       <c r="Q3" t="n">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
@@ -1263,16 +1263,16 @@
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>32.8</v>
+        <v>33.6</v>
       </c>
       <c r="Y3" t="n">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="Z3" t="n">
-        <v>50</v>
+        <v>53.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="AB3" t="n">
         <v>76.2</v>
@@ -1300,55 +1300,55 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>80</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D4" t="n">
-        <v>83.3</v>
+        <v>46.7</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F4" t="n">
-        <v>57.1</v>
+        <v>50</v>
       </c>
       <c r="G4" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="H4" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>43.2</v>
+        <v>23.8</v>
       </c>
       <c r="M4" t="n">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="N4" t="n">
-        <v>64.3</v>
+        <v>25</v>
       </c>
       <c r="O4" t="n">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="P4" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="Q4" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="R4" t="n">
-        <v>28.2</v>
+        <v>41</v>
       </c>
       <c r="S4" t="n">
         <v>39</v>
@@ -1363,16 +1363,16 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>28</v>
+        <v>43.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="Z4" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="AA4" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="AB4" t="n">
         <v>28.6</v>
@@ -1484,29 +1484,50 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>94.7</v>
+      </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="D6" t="n">
+        <v>78.90000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="F6" t="n">
+        <v>55.6</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
+      <c r="J6" t="n">
+        <v>66.7</v>
+      </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="L6" t="n">
+        <v>46.9</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>49</v>
+      </c>
+      <c r="N6" t="n">
+        <v>44</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="P6" t="n">
+        <v>20</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -1517,11 +1538,17 @@
       <c r="W6" t="n">
         <v>0</v>
       </c>
+      <c r="X6" t="n">
+        <v>70</v>
+      </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>33.3</v>
       </c>
       <c r="AA6" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -1540,88 +1567,88 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>71.7</v>
+        <v>73</v>
       </c>
       <c r="C7" t="n">
-        <v>205</v>
+        <v>248</v>
       </c>
       <c r="D7" t="n">
-        <v>57.7</v>
+        <v>56.9</v>
       </c>
       <c r="E7" t="n">
-        <v>537</v>
+        <v>624</v>
       </c>
       <c r="F7" t="n">
-        <v>66.7</v>
+        <v>63.1</v>
       </c>
       <c r="G7" t="n">
+        <v>195</v>
+      </c>
+      <c r="H7" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>545</v>
+      </c>
+      <c r="J7" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="K7" t="n">
+        <v>177</v>
+      </c>
+      <c r="L7" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="M7" t="n">
+        <v>435</v>
+      </c>
+      <c r="N7" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="O7" t="n">
         <v>162</v>
       </c>
-      <c r="H7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="I7" t="n">
-        <v>539</v>
-      </c>
-      <c r="J7" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="K7" t="n">
-        <v>148</v>
-      </c>
-      <c r="L7" t="n">
-        <v>19</v>
-      </c>
-      <c r="M7" t="n">
-        <v>300</v>
-      </c>
-      <c r="N7" t="n">
-        <v>22.6</v>
-      </c>
-      <c r="O7" t="n">
-        <v>93</v>
-      </c>
       <c r="P7" t="n">
-        <v>19.4</v>
+        <v>18.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>2826</v>
+        <v>3031</v>
       </c>
       <c r="R7" t="n">
-        <v>24.6</v>
+        <v>30.5</v>
       </c>
       <c r="S7" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="T7" t="n">
-        <v>32.1</v>
+        <v>31.2</v>
       </c>
       <c r="U7" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="V7" t="n">
-        <v>48.8</v>
+        <v>47.6</v>
       </c>
       <c r="W7" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="X7" t="n">
-        <v>36.2</v>
+        <v>40.1</v>
       </c>
       <c r="Y7" t="n">
-        <v>517</v>
+        <v>549</v>
       </c>
       <c r="Z7" t="n">
-        <v>52.4</v>
+        <v>52.3</v>
       </c>
       <c r="AA7" t="n">
-        <v>168</v>
+        <v>199</v>
       </c>
       <c r="AB7" t="n">
-        <v>61.6</v>
+        <v>61.2</v>
       </c>
       <c r="AC7" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="AD7" t="n">
         <v>100</v>

</xml_diff>